<commit_message>
docs(context): update stakeholder matrix (Excel artifact)
</commit_message>
<xml_diff>
--- a/docs/context-analysis/Stakeholder Matrix v1.0_Sawaka.xlsx
+++ b/docs/context-analysis/Stakeholder Matrix v1.0_Sawaka.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8da66447061942fd/Documents/sawaka/Documents/Business Analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berda\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{5864E17F-1BBB-6047-B5B2-02E3C641B246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{247712AF-379B-46A9-8712-57A6165E2B4C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C625BBF5-A68F-4E36-84C3-8ABB524747AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Stakeholder Matrix" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Z_015CA247_7A44_4B1F_B682_ED561B1AB267_.wvu.FilterData" localSheetId="0" hidden="1">'Stakeholder Matrix'!$A$4:$E$4</definedName>
+    <definedName name="Z_015CA247_7A44_4B1F_B682_ED561B1AB267_.wvu.FilterData" localSheetId="0" hidden="1">'Stakeholder Matrix'!$A$3:$E$3</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
@@ -31,7 +31,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="D4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -64,7 +64,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -97,7 +97,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="F3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -136,10 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="79">
-  <si>
-    <t>Use this stakeholder matrix to list of the stakeholders that are impacted or have influence over the project.</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="78">
   <si>
     <t>Prepared by:</t>
   </si>
@@ -439,7 +436,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -450,14 +447,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -540,7 +529,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -551,12 +540,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF9FC5E8"/>
         <bgColor rgb="FF9FC5E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEFEFEF"/>
-        <bgColor rgb="FFEFEFEF"/>
       </patternFill>
     </fill>
     <fill>
@@ -654,35 +637,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -901,7 +882,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.88671875" customWidth="1"/>
@@ -914,394 +895,392 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="5"/>
-    </row>
-    <row r="2" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-    </row>
-    <row r="3" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="E2" s="4">
+        <v>46059</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="B3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="9">
-        <v>46059</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>3</v>
+        <v>76</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>14</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="E4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="15" t="s">
+    </row>
+    <row r="9" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="15" t="s">
+      <c r="G9" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="15" t="s">
+      <c r="G10" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="E12" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="15" t="s">
+      <c r="G15" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9" s="15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="15" t="s">
+      <c r="G16" s="10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="G11" s="15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F16" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="G16" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="B17" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F17" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="G17" s="15" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="C18" s="15" t="s">
+      <c r="E17" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18" s="15" t="s">
+      <c r="G17" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="G18" s="15" t="s">
-        <v>76</v>
-      </c>
+    </row>
+    <row r="18" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
     </row>
     <row r="19" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
     </row>
     <row r="20" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
@@ -1312,25 +1291,15 @@
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
     </row>
-    <row r="21" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-    </row>
   </sheetData>
   <customSheetViews>
     <customSheetView guid="{015CA247-7A44-4B1F-B682-ED561B1AB267}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A4:E5" xr:uid="{0AE78201-8653-4E8A-8283-AE63BF22183C}"/>
+      <autoFilter ref="A4:E5" xr:uid="{91B21195-A9F0-46DE-8D83-D0DB1769252E}"/>
     </customSheetView>
   </customSheetViews>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>